<commit_message>
update RB module commit
</commit_message>
<xml_diff>
--- a/Log/Magic_eraser_test_log.xlsx
+++ b/Log/Magic_eraser_test_log.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23820" windowHeight="15380" firstSheet="3" activeTab="5"/>
+    <workbookView windowWidth="20320" windowHeight="16340" firstSheet="3" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Image_selector_test" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1057" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1094" uniqueCount="493">
   <si>
     <t>TC</t>
   </si>
@@ -1546,7 +1546,7 @@
     <t>Background flow</t>
   </si>
   <si>
-    <t>Preview Frame</t>
+    <t>Preview Frame (UI)</t>
   </si>
   <si>
     <t>- Ảnh được chọn trước đó đã được xử lý xong ở Processing flow
@@ -1554,7 +1554,137 @@
   </si>
   <si>
     <t>1. Mở màn hình Background 
-2. Quan sát sát khung preview</t>
+2. Quan sát khung preview cutout: 
++ Bo góc, tỷ lệ ảnh, không méo, không overflow 
++ Kiểm tra nút Cutout nằm đúng vị trí, icon + text đúng style 
+3. Kiểm tra các section title: 
++ font, size, alignment, spacing với các element khác 
+4. Kiểm tra section "Classics": 
++ Kích thước, bo góc, spacing (gap) đều 
++ Ảnh hiển thị đúng, không méo, không overflow 
+5. Cuộn xuống, kiểm tra section "Marketplaces" và section "Social" (các section có tác dụng resize): 
++ kích thước, bo góc, spacing (gap) đều 
++ border thể hiện đúng tỷ lệ hình ảnh sau thay đổi 
+6. Cuộn xuống cuối screen, kiểm rtra section Colors: 
++ kích thước, bo góc, spacing (gap) 
++ Màu nền background và vị trí vật thể 
+7. Kiểm tra section "Background Image": 
++ kích thước, bo góc, spacing (gap) 
++ hiển thị đúng thumnail thiết kế</t>
+  </si>
+  <si>
+    <t>- UI đúng theo thiết kế: font, maù, spacing, alignment. 
+- Preview frame hiển thị đugns, ảnh không méo, không overflow. 
+- Button Cutout đúng style và không bị tràn frame, nằm phía trên và không bị che đi bởi vật thể. 
+- Section titles đúng vị trí, font-size, spacing 
+- Tất cả các thumbnail hiển thị đúng kích thước 
+- Text lable dưới thumnail không bị crop hoặc overflow. 
+- Scroll mượt, không giật, không bị hiển thị rỗng 
+- Layout ổn định và không bị vỡ với các kích thước màn hình</t>
+  </si>
+  <si>
+    <t>RB_B_UI_02</t>
+  </si>
+  <si>
+    <t>Preview popup image selector ở section Background Image</t>
+  </si>
+  <si>
+    <t>- Ảnh được chọn trước đó đã được xử lý xong ở Processing flow 
+- Màn hình Background đã được load đầy đủ</t>
+  </si>
+  <si>
+    <t>1. Mở màn hình Background 
+2. Cuộng xuống cuối trang 
+3. chọn 1 thumnail thuộc nhóm "Background Image" 
+4. kiểm tra Popup "image selector": 
+- heading title hiển thị đúng font, font-size, spacing
+- cuộn lên xuống 
+- kích thước, bo góc, spacing của các image</t>
+  </si>
+  <si>
+    <t>- UI đúng theo thiết kế: font, màu, spacing, alignment
+- heading title đúng font, font-size, spacing so với thiết kế 
+- scroll mượt mà 
+- image đúng kích thước, bo góc, spacing, không bị over flow 
+- Layout ổn định và không bị thay đổi với các kích thước màn hình khác nhau</t>
+  </si>
+  <si>
+    <t>RB_BE_UI_ 01</t>
+  </si>
+  <si>
+    <t>Background-Edit flow</t>
+  </si>
+  <si>
+    <t>Preview popup main function</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Ở màn hình Background 
+- Ảnh đã được load thành công sau khi tách nền </t>
+  </si>
+  <si>
+    <t>1. Chọn 1 option (thumnail) ngẫu nhiên -&gt; Mở màn hình Edit background 
+2. Quan sát popup xuất hiện gồm 3 tabb: Size, Color, Image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Popup xuất hiện ở cạnh dưới màn hình
+- Layout, spacing, boder-radious, color, của các component đúng theo thiết kế 
+- Các nút cách đều không bị đè lên nhau </t>
+  </si>
+  <si>
+    <t>RB_BE_UI_02</t>
+  </si>
+  <si>
+    <t>Preview popup Size &amp; thumnail</t>
+  </si>
+  <si>
+    <t>- Ở màn Background-Edit 
+- Ảnh đã được load thành công sau khi chọn option</t>
+  </si>
+  <si>
+    <t>1. Chọn button "Size" để mở popup chức năng resize 
+2. Quan sát popup xuất hiện, kiểm tra kích thước hình dạng của border option đặc biệt tỷ lệ 2 cạnh, Logo biểu tượng, text lable, padding, spacing,  size text lable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Hiển thị đầy đủ danh sách template 
+- Mỗi template gồm: 
++ Icon/logo đúng theo nền tảng 
++ Tên template căn giữa, không bị tràn chữ 
++ Preview frame hiển thị đúng tý lệ (chiều dài/chiều rộng) 
+- Danh sách có thể scroll ngang 1 cách mượt mà 
+- buton "V","X" hiển thi đúng vị trí 2 bên góc, đúng size và spacing so với các component khác 
+- Template được chọn thì border sẽ đổi màu sang màu đỏ, các template còn lại có border
+- Text Lable cập nhật khi chọn các template khác nhau, hiển thị đúng font, font-size, nằm ở chính giữa đúng với thiết kế </t>
+  </si>
+  <si>
+    <t>RB_BE_UI_03</t>
+  </si>
+  <si>
+    <t>Preview popup Color &amp; thumnail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Ở màn Background-Edit 
+- Ảnh đã được load thành công sau khi chọn option </t>
+  </si>
+  <si>
+    <t>1. chọn buttonn "Color" để mở popup chức năng color 
+2. Kiểm tra Popup xuất hiện, kiểm tra kích thước, hình dạng của các thumnail 
+3. chọn thumnail custom color 
+4. Kiểm tra các component trong popup custom color: thanh mode màu, grid chọn màu, Bảng màu trong Spectrum, slider và input trong Sliders, Ô màu và các thumnail màu phí dưới</t>
+  </si>
+  <si>
+    <t>- Hiển thị đầy đủ dnah sách template 
+- với 2 thumnail none và custom color hiển thị đúng icon, padding của thiết kế 
+- các thumnail màu đơn sắc hiển thị đầy đủ, đúng kích thước và spacing, khi chọn vào các thumnail đơn sắc thì thumnail được chọn có dấu "V", các thumnail còn lại thì không 
+-  các component trong popup custom color hiển thị đúng padding, spacing, font, font-size so với thiết kế. 
+- ở nhóm Slider, các thanh màu sẽ tự động thay đổi theo màu sắc mà người dùng sẽ đạt được khi kéo thả các thanh slider
+- scroll ngang mượt
+- Không bị vỡ hay thay đổi layout với các kích thước màn hình khác nhau</t>
+  </si>
+  <si>
+    <t>RB_BE_UI_04</t>
+  </si>
+  <si>
+    <t>Preview popup Image &amp; thumnail</t>
   </si>
 </sst>
 </file>
@@ -7283,16 +7413,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="4"/>
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
-    <col min="1" max="1" width="6.640625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="21.09375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="18.359375" style="3" customWidth="1"/>
+    <col min="1" max="1" width="4.6875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="11.578125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="15.359375" style="3" customWidth="1"/>
     <col min="4" max="4" width="20.8359375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="28.8984375" style="3" customWidth="1"/>
-    <col min="6" max="6" width="24.4765625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="27.59375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="39.0625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="31.8984375" style="3" customWidth="1"/>
+    <col min="7" max="7" width="22" style="3" customWidth="1"/>
     <col min="8" max="8" width="10.6796875" style="3" customWidth="1"/>
     <col min="9" max="9" width="18.6171875" style="3" customWidth="1"/>
     <col min="10" max="10" width="20.953125" style="3" customWidth="1"/>
@@ -7362,7 +7492,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="3" ht="202" spans="1:13">
+    <row r="3" ht="168" spans="1:13">
       <c r="A3" s="3" t="s">
         <v>451</v>
       </c>
@@ -7384,7 +7514,6 @@
       <c r="G3" s="3" t="s">
         <v>457</v>
       </c>
-      <c r="H3" s="3"/>
       <c r="K3" s="3" t="s">
         <v>258</v>
       </c>
@@ -7395,7 +7524,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="4" ht="202" spans="1:7">
+    <row r="4" ht="168" spans="1:13">
       <c r="A4" s="3" t="s">
         <v>458</v>
       </c>
@@ -7417,8 +7546,17 @@
       <c r="G4" s="3" t="s">
         <v>463</v>
       </c>
-    </row>
-    <row r="5" ht="84" spans="1:5">
+      <c r="K4" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="5" ht="391" customHeight="1" spans="1:13">
       <c r="A5" s="3" t="s">
         <v>464</v>
       </c>
@@ -7433,6 +7571,124 @@
       </c>
       <c r="E5" s="3" t="s">
         <v>468</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>469</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="K5" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="M5" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="168" spans="1:13">
+      <c r="A6" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="D6" s="32" t="s">
+        <v>472</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="F6" s="32" t="s">
+        <v>474</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="7" ht="118" spans="1:6">
+      <c r="A7" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="D7" s="32" t="s">
+        <v>478</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="F7" s="32" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="8" ht="320" spans="1:6">
+      <c r="A8" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="D8" s="32" t="s">
+        <v>483</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="F8" s="32" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="9" ht="320" spans="1:6">
+      <c r="A9" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="D9" s="32" t="s">
+        <v>488</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="F9" s="32" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="10" ht="84" spans="1:4">
+      <c r="A10" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="D10" s="32" t="s">
+        <v>488</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finish test case Remove background
</commit_message>
<xml_diff>
--- a/Log/Magic_eraser_test_log.xlsx
+++ b/Log/Magic_eraser_test_log.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20320" windowHeight="16340" firstSheet="3" activeTab="5"/>
+    <workbookView windowWidth="25820" windowHeight="16340" firstSheet="3" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Image_selector_test" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1094" uniqueCount="493">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1112" uniqueCount="500">
   <si>
     <t>TC</t>
   </si>
@@ -1554,30 +1554,19 @@
   </si>
   <si>
     <t>1. Mở màn hình Background 
-2. Quan sát khung preview cutout: 
-+ Bo góc, tỷ lệ ảnh, không méo, không overflow 
-+ Kiểm tra nút Cutout nằm đúng vị trí, icon + text đúng style 
-3. Kiểm tra các section title: 
-+ font, size, alignment, spacing với các element khác 
-4. Kiểm tra section "Classics": 
-+ Kích thước, bo góc, spacing (gap) đều 
-+ Ảnh hiển thị đúng, không méo, không overflow 
-5. Cuộn xuống, kiểm tra section "Marketplaces" và section "Social" (các section có tác dụng resize): 
-+ kích thước, bo góc, spacing (gap) đều 
-+ border thể hiện đúng tỷ lệ hình ảnh sau thay đổi 
-6. Cuộn xuống cuối screen, kiểm rtra section Colors: 
-+ kích thước, bo góc, spacing (gap) 
-+ Màu nền background và vị trí vật thể 
-7. Kiểm tra section "Background Image": 
-+ kích thước, bo góc, spacing (gap) 
-+ hiển thị đúng thumnail thiết kế</t>
+2. Quan sát khung preview cutout
+3. Kiểm tra các section title
+4. Kiểm tra section "Classics"
+5. Cuộn xuống, kiểm tra section "Marketplaces" và section "Social" (các section có tác dụng resize)
+6. Cuộn xuống cuối screen, kiểm rtra section Colors
+7. Kiểm tra section "Background Image"</t>
   </si>
   <si>
     <t>- UI đúng theo thiết kế: font, maù, spacing, alignment. 
 - Preview frame hiển thị đugns, ảnh không méo, không overflow. 
 - Button Cutout đúng style và không bị tràn frame, nằm phía trên và không bị che đi bởi vật thể. 
 - Section titles đúng vị trí, font-size, spacing 
-- Tất cả các thumbnail hiển thị đúng kích thước 
+- Tất cả các thumbnail hiển thị đúng kích thước (đối với thumnail thuộc section "Marketplaces" &amp; "Social" thì thể hiện đúng tỷ lệ cạnh mà ảnh sẽ thay đổi sau khi chọn thumnail đó) 
 - Text lable dưới thumnail không bị crop hoặc overflow. 
 - Scroll mượt, không giật, không bị hiển thị rỗng 
 - Layout ổn định và không bị vỡ với các kích thước màn hình</t>
@@ -1597,7 +1586,7 @@
 2. Cuộng xuống cuối trang 
 3. chọn 1 thumnail thuộc nhóm "Background Image" 
 4. kiểm tra Popup "image selector": 
-- heading title hiển thị đúng font, font-size, spacing
+- quan sát heading title
 - cuộn lên xuống 
 - kích thước, bo góc, spacing của các image</t>
   </si>
@@ -1648,7 +1637,7 @@
     <t xml:space="preserve">- Hiển thị đầy đủ danh sách template 
 - Mỗi template gồm: 
 + Icon/logo đúng theo nền tảng 
-+ Tên template căn giữa, không bị tràn chữ 
++ Tên template căn giữa, không bị tràn chữ, nếu tên dài thì trình bày xuống 2 dòng (font-size thống nhất)
 + Preview frame hiển thị đúng tý lệ (chiều dài/chiều rộng) 
 - Danh sách có thể scroll ngang 1 cách mượt mà 
 - buton "V","X" hiển thi đúng vị trí 2 bên góc, đúng size và spacing so với các component khác 
@@ -1672,7 +1661,7 @@
 4. Kiểm tra các component trong popup custom color: thanh mode màu, grid chọn màu, Bảng màu trong Spectrum, slider và input trong Sliders, Ô màu và các thumnail màu phí dưới</t>
   </si>
   <si>
-    <t>- Hiển thị đầy đủ dnah sách template 
+    <t>- Hiển thị đầy đủ danh sách template 
 - với 2 thumnail none và custom color hiển thị đúng icon, padding của thiết kế 
 - các thumnail màu đơn sắc hiển thị đầy đủ, đúng kích thước và spacing, khi chọn vào các thumnail đơn sắc thì thumnail được chọn có dấu "V", các thumnail còn lại thì không 
 -  các component trong popup custom color hiển thị đúng padding, spacing, font, font-size so với thiết kế. 
@@ -1685,6 +1674,67 @@
   </si>
   <si>
     <t>Preview popup Image &amp; thumnail</t>
+  </si>
+  <si>
+    <t>1. Chọn button "Image" để mở popup chức năng chèn ảnh 
+2. Kiểm tra layout và alignment của popup, sau đó kiểm tra riêng các component trong popup: 
+2.a. kiểm tra topic lable bar
+2.b. kiểm tra thumnail bar 
+3. scroll ngang topic bar và thumnail bar 
+4. chọn topic lable và thumnail và kiểm tra hiệu ứng khi chọn của chúng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Hiển thị đầy đủ danh sách topic, thumnail 
+- với 2 thumnail None và upload image hiển thị đúng icon, pading đúng với thiết kế 
+- các thumnail hình ảnh có sẵn hiển thị đầy đủ, đúng size và spacing, giữa các nhóm thumnail thuộc các topic khác nhau  có đường kẻ chia cách chúng 
+- Topic lable hiển thị đúng font, font-size, spacing. 
+- Topic lable được chọn có font-color và underline màu đỏ
+- Thumnail được chọn có boder được tô đỏ.
+- khi chọn 1 topic lable thì scroll đến thumnail đầu tiên của nhóm thumnail thuộc topic đó.
+- scroll ngang mượt, không giật, hay nhảy cóc 
+- Layout ổn định, không bị vỡ hay ép với các kích thước màn hình khác nhau </t>
+  </si>
+  <si>
+    <t>RB_BE_F_01</t>
+  </si>
+  <si>
+    <t>Background editting flow (quá trình chỉnh sửa - edit phông nền)</t>
+  </si>
+  <si>
+    <t>- Ở màn hình Background 
+- Ảnh đã được xử lý tách nền thành công</t>
+  </si>
+  <si>
+    <t>1. Chọn một thumbnail background bất kỳ để áp dụng. 
+2. Di chuyển vị trí vật thể trên ảnh 
+3. Mở công cụ Resize, thao tác thử các lựa chọn resize.
+4. Mở công cụ Color, lần lượt thao tác các chức năng:
++ Chọn màu đơn có sẵn
++ Chọn màu tùy chỉnh (grid, spectrum)
++ Điều chỉnh sắc độ hoặc nhập mã màu (RGB/Hex)
++ Trích xuất màu từ hình ảnh
++ Thêm màu mới và chọn lại màu vừa thêm
+5. Mở công cụ Image, thực hiện các thao tác:
++ Upload ảnh từ thiết bị
++ Chọn template (topic label)
++ Chọn nhiều thumbnail khác nhau
+6. Thực hiện thao tác Undo/Redo hoặc Reset chỉnh sửa.
+7. Nhấn Save để lưu hình ảnh.</t>
+  </si>
+  <si>
+    <t>- Mở màn hình Background-Edit: 
++ button undo và redo bị vô hiệu khi không có thao tác chỉnh sửa nào đã được thực hiện 
++ layer vật thể được tách nền được chọn (bo khung đỏ)
++ popup chức năng chính bao gồm 3 button chức năng lớn: Size, Color, Image
+- Khi vật thể dịch chuyển theo thao tác người dùng, Khi thả ra thì hệ thống ghi nhận 1 thao tác chỉnh sửa 
+- Các pop-up chức năng hiển thị đúng với lựa chọn (Size, Color, Image) 
+- Các chức năng con hoạt động đúng: 
++ Size: kích thước ảnh thay đổi theo lựa chọn, phần text lable cập nhật đúng theo kích thước được chọn 
++ Color: Các template color cho sẵn và template trong suốt hoạt động đúng; Custom color hoặt động đúng, có thể lưu màu mới custom, ảnh được cập nhật màu theo màu đang custom. 
++ Image: topic bar scoll mượt mà, khi 1 topic được chọn thì chuyển sang màu đỏ và thumnail bar được scroll đến thumnail đầu tiên thuộc topic đó; option chọn được viền đỏ và background preview được cập nhật 
+- Undo/redo và reset hoạt động đúng logic 
+- Có thể phóng to, thu nhỏ và xoay vật thể (layer)
+- Ảnh được lưu vào máy đúng với kết quả chỉnh sửa và chuyển sang màn hình saved</t>
   </si>
 </sst>
 </file>
@@ -7413,16 +7463,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="4.6875" style="3" customWidth="1"/>
     <col min="2" max="2" width="11.578125" style="3" customWidth="1"/>
     <col min="3" max="3" width="15.359375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="20.8359375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="39.0625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="31.8984375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="22" style="3" customWidth="1"/>
+    <col min="4" max="4" width="19.3984375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="35.15625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="51.296875" style="3" customWidth="1"/>
+    <col min="7" max="7" width="17.96875" style="3" customWidth="1"/>
     <col min="8" max="8" width="10.6796875" style="3" customWidth="1"/>
     <col min="9" max="9" width="18.6171875" style="3" customWidth="1"/>
     <col min="10" max="10" width="20.953125" style="3" customWidth="1"/>
@@ -7492,7 +7542,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="3" ht="168" spans="1:13">
+    <row r="3" ht="152" spans="1:13">
       <c r="A3" s="3" t="s">
         <v>451</v>
       </c>
@@ -7524,7 +7574,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="4" ht="168" spans="1:13">
+    <row r="4" ht="118" spans="1:13">
       <c r="A4" s="3" t="s">
         <v>458</v>
       </c>
@@ -7556,7 +7606,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="5" ht="391" customHeight="1" spans="1:13">
+    <row r="5" ht="193" customHeight="1" spans="1:13">
       <c r="A5" s="3" t="s">
         <v>464</v>
       </c>
@@ -7588,7 +7638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" ht="168" spans="1:13">
+    <row r="6" ht="152" spans="1:13">
       <c r="A6" s="3" t="s">
         <v>470</v>
       </c>
@@ -7617,7 +7667,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="7" ht="118" spans="1:6">
+    <row r="7" ht="84" spans="1:6">
       <c r="A7" s="3" t="s">
         <v>475</v>
       </c>
@@ -7637,7 +7687,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="8" ht="320" spans="1:6">
+    <row r="8" ht="224" customHeight="1" spans="1:13">
       <c r="A8" s="3" t="s">
         <v>481</v>
       </c>
@@ -7656,8 +7706,17 @@
       <c r="F8" s="32" t="s">
         <v>485</v>
       </c>
-    </row>
-    <row r="9" ht="320" spans="1:6">
+      <c r="K8" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="9" ht="219" spans="1:6">
       <c r="A9" s="3" t="s">
         <v>486</v>
       </c>
@@ -7677,7 +7736,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="10" ht="84" spans="1:4">
+    <row r="10" ht="236" spans="1:13">
       <c r="A10" s="3" t="s">
         <v>491</v>
       </c>
@@ -7689,6 +7748,53 @@
       </c>
       <c r="D10" s="32" t="s">
         <v>488</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="F10" s="32" t="s">
+        <v>494</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="11" ht="409" customHeight="1" spans="1:13">
+      <c r="A11" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="D11" s="32" t="s">
+        <v>497</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="F11" s="32" t="s">
+        <v>499</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RB test tescase update
</commit_message>
<xml_diff>
--- a/Log/Magic_eraser_test_log.xlsx
+++ b/Log/Magic_eraser_test_log.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25820" windowHeight="16340" firstSheet="3" activeTab="5"/>
+    <workbookView windowWidth="27320" windowHeight="10920" firstSheet="3" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Image_selector_test" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1112" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1115" uniqueCount="500">
   <si>
     <t>TC</t>
   </si>
@@ -1437,7 +1437,7 @@
     <t>Mã TC của Connect with us: CWU</t>
   </si>
   <si>
-    <t>Test cases: module Processing  (ID: PR)</t>
+    <t>Test cases: module Remove-Background  (ID: RB)</t>
   </si>
   <si>
     <t>Android</t>
@@ -1631,7 +1631,7 @@
   </si>
   <si>
     <t>1. Chọn button "Size" để mở popup chức năng resize 
-2. Quan sát popup xuất hiện, kiểm tra kích thước hình dạng của border option đặc biệt tỷ lệ 2 cạnh, Logo biểu tượng, text lable, padding, spacing,  size text lable</t>
+2. Quan sát popup xuất hiện, kiểm tra UI</t>
   </si>
   <si>
     <t xml:space="preserve">- Hiển thị đầy đủ danh sách template 
@@ -1642,6 +1642,7 @@
 - Danh sách có thể scroll ngang 1 cách mượt mà 
 - buton "V","X" hiển thi đúng vị trí 2 bên góc, đúng size và spacing so với các component khác 
 - Template được chọn thì border sẽ đổi màu sang màu đỏ, các template còn lại có border
+- Template không đè lên và che đi phần preview hình ảnh
 - Text Lable cập nhật khi chọn các template khác nhau, hiển thị đúng font, font-size, nằm ở chính giữa đúng với thiết kế </t>
   </si>
   <si>
@@ -7667,7 +7668,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="7" ht="84" spans="1:6">
+    <row r="7" ht="84" spans="1:13">
       <c r="A7" s="3" t="s">
         <v>475</v>
       </c>
@@ -7686,8 +7687,17 @@
       <c r="F7" s="32" t="s">
         <v>480</v>
       </c>
-    </row>
-    <row r="8" ht="224" customHeight="1" spans="1:13">
+      <c r="K7" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="8" ht="245" customHeight="1" spans="1:13">
       <c r="A8" s="3" t="s">
         <v>481</v>
       </c>

</xml_diff>

<commit_message>
new test case commit
</commit_message>
<xml_diff>
--- a/Log/Magic_eraser_test_log.xlsx
+++ b/Log/Magic_eraser_test_log.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27320" windowHeight="10920" firstSheet="3" activeTab="5"/>
+    <workbookView windowHeight="15700" firstSheet="3" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Image_selector_test" sheetId="1" r:id="rId1"/>
@@ -1214,7 +1214,7 @@
 6. chọn button Less</t>
   </si>
   <si>
-    <t>Chuyển tiếp mượt mà giữa các màn: màn giới thiệu chức năng, màn thăm dò, màn tiếp thị, màn Home. Nhấn nút More sẽ hiển thị toàn bộ các button chức năng, nút Lesss ẩn bớt các chức năng</t>
+    <t>Chuyển tiếp mượt mà giữa các màn: màn "fearture introduction" -&gt; màn thăm dò -&gt; màn "Payment" -&gt; màn "Home". Nhấn nút More sẽ hiển thị toàn bộ các button chức năng, nút Lesss ẩn bớt các chức năng</t>
   </si>
   <si>
     <t>BE</t>
@@ -7177,7 +7177,7 @@
       </c>
       <c r="I1" s="5"/>
     </row>
-    <row r="2" ht="159" customHeight="1" spans="1:9">
+    <row r="2" ht="182" customHeight="1" spans="1:9">
       <c r="A2" s="5" t="s">
         <v>382</v>
       </c>

</xml_diff>